<commit_message>
Present mode: letterboxed 16:9, chrome hidden by default; expand polling rationale
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/workshop/DEV-TRACKER.xlsx
+++ b/docs/workshop/DEV-TRACKER.xlsx
@@ -2048,7 +2048,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2596,440 +2596,471 @@
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
+          <t>T2.9</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Present default chrome-free</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>Open present mode fresh in windows of several aspect ratios; move mouse; press T/N; pin the timer; go idle 3s</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>Only the slide visible, letterboxed 16:9 on black; overlays appear on mouse/hotkey and auto-hide ~3s; pinned timer stays</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>Untested</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
           <t>T3.1</t>
         </is>
       </c>
-      <c r="B18" s="8" t="n">
+      <c r="B19" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>Graceful no-key state</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr">
         <is>
           <t>Unset ANTHROPIC_API_KEY; open generation dialog</t>
         </is>
       </c>
-      <c r="E18" s="8" t="inlineStr">
+      <c r="E19" s="8" t="inlineStr">
         <is>
           <t>Clear 'AI unavailable' message; rest of app fully functional</t>
         </is>
       </c>
-      <c r="F18" s="8" t="inlineStr">
+      <c r="F19" s="8" t="inlineStr">
         <is>
           <t>Untested</t>
         </is>
       </c>
-      <c r="G18" s="8" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="9" t="inlineStr">
+      <c r="G19" s="8" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
         <is>
           <t>T3.2</t>
         </is>
       </c>
-      <c r="B19" s="9" t="n">
+      <c r="B20" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="C19" s="9" t="inlineStr">
+      <c r="C20" s="9" t="inlineStr">
         <is>
           <t>Generate slides</t>
         </is>
       </c>
-      <c r="D19" s="9" t="inlineStr">
+      <c r="D20" s="9" t="inlineStr">
         <is>
           <t>Generate 3 slides (bullets, big-number, debrief) for a real item; once with Vietnamese content</t>
         </is>
       </c>
-      <c r="E19" s="9" t="inlineStr">
+      <c r="E20" s="9" t="inlineStr">
         <is>
           <t>All validate against schemas, render without hand-fixing, correct language</t>
         </is>
       </c>
-      <c r="F19" s="9" t="inlineStr">
+      <c r="F20" s="9" t="inlineStr">
         <is>
           <t>Untested</t>
         </is>
       </c>
-      <c r="G19" s="9" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="G20" s="9" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>T3.3</t>
         </is>
       </c>
-      <c r="B20" s="8" t="n">
+      <c r="B21" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="C20" s="8" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>Regenerate with refinement</t>
         </is>
       </c>
-      <c r="D20" s="8" t="inlineStr">
+      <c r="D21" s="8" t="inlineStr">
         <is>
           <t>Regenerate one reviewed slide with a refinement instruction; accept</t>
         </is>
       </c>
-      <c r="E20" s="8" t="inlineStr">
+      <c r="E21" s="8" t="inlineStr">
         <is>
           <t>Only that slide changes; accepted slide attached to right item in order</t>
         </is>
       </c>
-      <c r="F20" s="8" t="inlineStr">
+      <c r="F21" s="8" t="inlineStr">
         <is>
           <t>Untested</t>
         </is>
       </c>
-      <c r="G20" s="8" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="9" t="inlineStr">
+      <c r="G21" s="8" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
         <is>
           <t>T3.4</t>
         </is>
       </c>
-      <c r="B21" s="9" t="n">
+      <c r="B22" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="C21" s="9" t="inlineStr">
+      <c r="C22" s="9" t="inlineStr">
         <is>
           <t>Edit-via-prompt precision</t>
         </is>
       </c>
-      <c r="D21" s="9" t="inlineStr">
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t>Ask to change one aspect of an existing slide</t>
         </is>
       </c>
-      <c r="E21" s="9" t="inlineStr">
+      <c r="E22" s="9" t="inlineStr">
         <is>
           <t>Exactly the requested aspect changes in fields</t>
         </is>
       </c>
-      <c r="F21" s="9" t="inlineStr">
+      <c r="F22" s="9" t="inlineStr">
         <is>
           <t>Untested</t>
         </is>
       </c>
-      <c r="G21" s="9" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="8" t="inlineStr">
+      <c r="G22" s="9" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>T3.5</t>
         </is>
       </c>
-      <c r="B22" s="8" t="n">
+      <c r="B23" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="C22" s="8" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>Generate template</t>
         </is>
       </c>
-      <c r="D22" s="8" t="inlineStr">
+      <c r="D23" s="8" t="inlineStr">
         <is>
           <t>Describe 'myth vs fact two-panel with reveal'</t>
         </is>
       </c>
-      <c r="E22" s="8" t="inlineStr">
+      <c r="E23" s="8" t="inlineStr">
         <is>
           <t>Draft previews with sample data; after save usable on a new slide</t>
         </is>
       </c>
-      <c r="F22" s="8" t="inlineStr">
+      <c r="F23" s="8" t="inlineStr">
         <is>
           <t>Untested</t>
         </is>
       </c>
-      <c r="G22" s="8" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="9" t="inlineStr">
+      <c r="G23" s="8" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
         <is>
           <t>T3.6</t>
         </is>
       </c>
-      <c r="B23" s="9" t="n">
+      <c r="B24" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="C23" s="9" t="inlineStr">
+      <c r="C24" s="9" t="inlineStr">
         <is>
           <t>Caps + logging</t>
         </is>
       </c>
-      <c r="D23" s="9" t="inlineStr">
+      <c r="D24" s="9" t="inlineStr">
         <is>
           <t>Set cap override to 2; make 3 calls; check /usage</t>
         </is>
       </c>
-      <c r="E23" s="9" t="inlineStr">
+      <c r="E24" s="9" t="inlineStr">
         <is>
           <t>Third call → 429 surfaced politely; tokens logged in ai_generations; usage sums match</t>
         </is>
       </c>
-      <c r="F23" s="9" t="inlineStr">
+      <c r="F24" s="9" t="inlineStr">
         <is>
           <t>Untested</t>
         </is>
       </c>
-      <c r="G23" s="9" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="8" t="inlineStr">
+      <c r="G24" s="9" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>T4.1</t>
         </is>
       </c>
-      <c r="B24" s="8" t="n">
+      <c r="B25" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="C24" s="8" t="inlineStr">
+      <c r="C25" s="8" t="inlineStr">
         <is>
           <t>Session join</t>
         </is>
       </c>
-      <c r="D24" s="8" t="inlineStr">
+      <c r="D25" s="8" t="inlineStr">
         <is>
           <t>Start session; scan QR with a real phone</t>
         </is>
       </c>
-      <c r="E24" s="8" t="inlineStr">
+      <c r="E25" s="8" t="inlineStr">
         <is>
           <t>Code + QR on player; phone joins without login</t>
         </is>
       </c>
-      <c r="F24" s="8" t="inlineStr">
+      <c r="F25" s="8" t="inlineStr">
         <is>
           <t>Untested</t>
         </is>
       </c>
-      <c r="G24" s="8" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="9" t="inlineStr">
+      <c r="G25" s="8" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="inlineStr">
         <is>
           <t>T4.2</t>
         </is>
       </c>
-      <c r="B25" s="9" t="n">
+      <c r="B26" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="C25" s="9" t="inlineStr">
+      <c r="C26" s="9" t="inlineStr">
         <is>
           <t>Poll live round-trip</t>
         </is>
       </c>
-      <c r="D25" s="9" t="inlineStr">
+      <c r="D26" s="9" t="inlineStr">
         <is>
           <t>Activate poll; vote; re-vote; deactivate</t>
         </is>
       </c>
-      <c r="E25" s="9" t="inlineStr">
+      <c r="E26" s="9" t="inlineStr">
         <is>
           <t>Bar updates ≤2s; re-vote replaces (count unchanged); deactivate freezes results, phone shows waiting</t>
         </is>
       </c>
-      <c r="F25" s="9" t="inlineStr">
+      <c r="F26" s="9" t="inlineStr">
         <is>
           <t>Untested</t>
         </is>
       </c>
-      <c r="G25" s="9" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="8" t="inlineStr">
+      <c r="G26" s="9" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
         <is>
           <t>T4.3</t>
         </is>
       </c>
-      <c r="B26" s="8" t="n">
+      <c r="B27" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="C26" s="8" t="inlineStr">
+      <c r="C27" s="8" t="inlineStr">
         <is>
           <t>Word cloud + XSS probe</t>
         </is>
       </c>
-      <c r="D26" s="8" t="inlineStr">
+      <c r="D27" s="8" t="inlineStr">
         <is>
           <t>3+ phones submit words; one submits '&lt;img src=x onerror=alert(1)&gt;'</t>
         </is>
       </c>
-      <c r="E26" s="8" t="inlineStr">
+      <c r="E27" s="8" t="inlineStr">
         <is>
           <t>Cloud scales by frequency; probe renders as inert text (text nodes only)</t>
         </is>
       </c>
-      <c r="F26" s="8" t="inlineStr">
+      <c r="F27" s="8" t="inlineStr">
         <is>
           <t>Untested</t>
         </is>
       </c>
-      <c r="G26" s="8" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="9" t="inlineStr">
+      <c r="G27" s="8" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
         <is>
           <t>T4.4</t>
         </is>
       </c>
-      <c r="B27" s="9" t="n">
+      <c r="B28" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="C27" s="9" t="inlineStr">
+      <c r="C28" s="9" t="inlineStr">
         <is>
           <t>Quiz reveal</t>
         </is>
       </c>
-      <c r="D27" s="9" t="inlineStr">
+      <c r="D28" s="9" t="inlineStr">
         <is>
           <t>Run quiz slide: vote, then advance to reveal step</t>
         </is>
       </c>
-      <c r="E27" s="9" t="inlineStr">
+      <c r="E28" s="9" t="inlineStr">
         <is>
           <t>Votes hidden until reveal; reveal shows distribution + highlights correct answer</t>
         </is>
       </c>
-      <c r="F27" s="9" t="inlineStr">
+      <c r="F28" s="9" t="inlineStr">
         <is>
           <t>Untested</t>
         </is>
       </c>
-      <c r="G27" s="9" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="8" t="inlineStr">
+      <c r="G28" s="9" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
         <is>
           <t>T4.5</t>
         </is>
       </c>
-      <c r="B28" s="8" t="n">
+      <c r="B29" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="C28" s="8" t="inlineStr">
+      <c r="C29" s="8" t="inlineStr">
         <is>
           <t>Rating + hotspot kinds</t>
         </is>
       </c>
-      <c r="D28" s="8" t="inlineStr">
+      <c r="D29" s="8" t="inlineStr">
         <is>
           <t>Run rating and hotspot slides end-to-end on a phone</t>
         </is>
       </c>
-      <c r="E28" s="8" t="inlineStr">
+      <c r="E29" s="8" t="inlineStr">
         <is>
           <t>Both submit and render aggregates (avg+distribution; dot overlay)</t>
         </is>
       </c>
-      <c r="F28" s="8" t="inlineStr">
+      <c r="F29" s="8" t="inlineStr">
         <is>
           <t>Untested</t>
         </is>
       </c>
-      <c r="G28" s="8" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="9" t="inlineStr">
+      <c r="G29" s="8" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
         <is>
           <t>T4.6</t>
         </is>
       </c>
-      <c r="B29" s="9" t="n">
+      <c r="B30" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="C29" s="9" t="inlineStr">
+      <c r="C30" s="9" t="inlineStr">
         <is>
           <t>Snapshot isolation</t>
         </is>
       </c>
-      <c r="D29" s="9" t="inlineStr">
+      <c r="D30" s="9" t="inlineStr">
         <is>
           <t>Edit the workshop while a session is live</t>
         </is>
       </c>
-      <c r="E29" s="9" t="inlineStr">
+      <c r="E30" s="9" t="inlineStr">
         <is>
           <t>Live session unaffected (published snapshot)</t>
         </is>
       </c>
-      <c r="F29" s="9" t="inlineStr">
+      <c r="F30" s="9" t="inlineStr">
         <is>
           <t>Untested</t>
         </is>
       </c>
-      <c r="G29" s="9" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="8" t="inlineStr">
+      <c r="G30" s="9" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
         <is>
           <t>T4.7</t>
         </is>
       </c>
-      <c r="B30" s="8" t="n">
+      <c r="B31" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="C30" s="8" t="inlineStr">
+      <c r="C31" s="8" t="inlineStr">
         <is>
           <t>Load test</t>
         </is>
       </c>
-      <c r="D30" s="8" t="inlineStr">
+      <c r="D31" s="8" t="inlineStr">
         <is>
           <t>node scripts/workshop-participant-sim.js 30</t>
         </is>
       </c>
-      <c r="E30" s="8" t="inlineStr">
+      <c r="E31" s="8" t="inlineStr">
         <is>
           <t>Zero errors, counts correct, player stays smooth</t>
         </is>
       </c>
-      <c r="F30" s="8" t="inlineStr">
+      <c r="F31" s="8" t="inlineStr">
         <is>
           <t>Untested</t>
         </is>
       </c>
-      <c r="G30" s="8" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="9" t="inlineStr">
+      <c r="G31" s="8" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="9" t="inlineStr">
         <is>
           <t>T4.8</t>
         </is>
       </c>
-      <c r="B31" s="9" t="n">
+      <c r="B32" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="C31" s="9" t="inlineStr">
+      <c r="C32" s="9" t="inlineStr">
         <is>
           <t>Session end state</t>
         </is>
       </c>
-      <c r="D31" s="9" t="inlineStr">
+      <c r="D32" s="9" t="inlineStr">
         <is>
           <t>End session; open join page; open read mode</t>
         </is>
       </c>
-      <c r="E31" s="9" t="inlineStr">
+      <c r="E32" s="9" t="inlineStr">
         <is>
           <t>Join page says session ended; results still visible in read mode</t>
         </is>
       </c>
-      <c r="F31" s="9" t="inlineStr">
+      <c r="F32" s="9" t="inlineStr">
         <is>
           <t>Untested</t>
         </is>
       </c>
-      <c r="G31" s="9" t="inlineStr"/>
+      <c r="G32" s="9" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F2:F32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Untested,Pass,Fail,Blocked"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>